<commit_message>
Major importer and website updates
</commit_message>
<xml_diff>
--- a/imports/Test/test.xlsx
+++ b/imports/Test/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhwan\Desktop\sparesco-catalog\imports\Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB59D995-5C26-494F-8878-0B6120D058E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5138C988-BF11-4A02-9AFC-BDD8B9F00BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="168">
   <si>
     <t>Handle</t>
   </si>
@@ -187,307 +187,343 @@
     <t>Variant Metafield: custom.shipping_volume [single_line_text_field]</t>
   </si>
   <si>
+    <t>sa-18278</t>
+  </si>
+  <si>
+    <t>MERGE</t>
+  </si>
+  <si>
+    <t>SA 18278</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>web</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/md-ac85c596-affc-4f36-abe9-8de7752a4538.jpg?v=1723235210</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>HiFi Filter SA 18278 Air Filter</t>
+  </si>
+  <si>
+    <t>sa-18278-1</t>
+  </si>
+  <si>
+    <t>shopify</t>
+  </si>
+  <si>
+    <t>continue</t>
+  </si>
+  <si>
+    <t>manual</t>
+  </si>
+  <si>
+    <t>General Profile</t>
+  </si>
+  <si>
+    <t>8421.99.90</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Genuine HiFi Filter SA 18278 Air Filter. Easy to install and replace, the SA 18278 is built to withstand demanding environments, offering long-lasting protection and reliability. Whether used in automotive, agricultural, construction, or industrial applications, this filter is an essential component for maintaining system health and performance.</t>
+  </si>
+  <si>
+    <t>2.18 kg</t>
+  </si>
+  <si>
+    <t>0.0246 m³</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/AF26531.jpg?v=1755780998</t>
+  </si>
+  <si>
+    <t>Fleetguard AF26531 Air Filter, Primary | Replaces the HiFi Filter SA 18278</t>
+  </si>
+  <si>
+    <t>sa-18278-2</t>
+  </si>
+  <si>
+    <t>8421.31.00</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>​Fleetguard® AF26531 axial seal primary air filter ensures a proper seal and prevent leaks to prevent airborne contaminants from reaching the combustion chamber.</t>
+  </si>
+  <si>
+    <t>AF26531</t>
+  </si>
+  <si>
+    <t>2.24 kg</t>
+  </si>
+  <si>
+    <t>0.002 m³</t>
+  </si>
+  <si>
+    <t>8421.23.00</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>0.38 kg</t>
+  </si>
+  <si>
+    <t>Style: AIR FILTER, Dimension 1 (D1): 226.0 mm, Dimension 2 (D2): 183.0 mm, Dimension 3 (D3): 139.0 mm, Height 1 (H1): 379.0 mm, Height 2 (H2): 378.0 mm, Height 3 (H3): 30.0 mm</t>
+  </si>
+  <si>
+    <t>Style: Air Filter</t>
+  </si>
+  <si>
+    <t>Variant Metafield: custom.hs_code [single_line_text_field]</t>
+  </si>
+  <si>
+    <t>Variant Metafield: custom.country_of_origin [single_line_text_field]</t>
+  </si>
+  <si>
+    <t>0.34 kg</t>
+  </si>
+  <si>
+    <t>0.0008 m³</t>
+  </si>
+  <si>
+    <t>0.64 kg</t>
+  </si>
+  <si>
+    <t>0.73 kg</t>
+  </si>
+  <si>
+    <t>0.67 kg</t>
+  </si>
+  <si>
+    <t>0.0011 m³</t>
+  </si>
+  <si>
+    <t>0.0005 m³</t>
+  </si>
+  <si>
+    <t>0.0013 m³</t>
+  </si>
+  <si>
+    <t>0.0035 m³</t>
+  </si>
+  <si>
+    <t>0.15 kg</t>
+  </si>
+  <si>
+    <t>8421.29.80.90</t>
+  </si>
+  <si>
+    <t>United Kingdom</t>
+  </si>
+  <si>
+    <t>0.33 kg</t>
+  </si>
+  <si>
+    <t>Variant Metafield: custom.vendor [single_line_text_field]</t>
+  </si>
+  <si>
+    <t>Filter, ff1225, test</t>
+  </si>
+  <si>
     <t>he120-5</t>
   </si>
   <si>
-    <t>MERGE</t>
-  </si>
-  <si>
     <t>HE120 5</t>
   </si>
   <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>TRUE</t>
-  </si>
-  <si>
-    <t>web</t>
-  </si>
-  <si>
     <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/FF300404C_d07d8d17-8307-4491-ae53-82336df06ba7.jpg?v=1760959546</t>
   </si>
   <si>
-    <t>Brand</t>
-  </si>
-  <si>
     <t>FilterFinder FF300404C Compressed Air Filter | Replaces the Hi-Line HE120-5</t>
   </si>
   <si>
     <t>he120-5-1</t>
   </si>
   <si>
-    <t>shopify</t>
-  </si>
-  <si>
-    <t>continue</t>
-  </si>
-  <si>
-    <t>manual</t>
-  </si>
-  <si>
-    <t>General Profile</t>
-  </si>
-  <si>
     <t>Style: Compressed Air Filter, Media: Polyester Needle Felt, Outer Diameter: 76.0 mm, Inner Diameter: 41.0 mm, Length: 118.0 mm, Seal Material: Nitrile, Temperature Range: +1 - +80°C, Media Type: Polyester Needle Felt, Flow Direction: IN-OUT, Seal: Nitrile</t>
   </si>
   <si>
     <t>FF300404C</t>
   </si>
   <si>
-    <t>he120-3</t>
-  </si>
-  <si>
-    <t>HE120 3</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/FF300402C_c4f5417c-368a-4799-8be6-3435e4941c04.jpg?v=1760959543</t>
-  </si>
-  <si>
-    <t>FilterFinder FF300402C Compressed Air Filter | Replaces the Hi-Line HE120-3</t>
-  </si>
-  <si>
-    <t>he120-3-1</t>
-  </si>
-  <si>
-    <t>FF300402C</t>
-  </si>
-  <si>
-    <t>he50-3</t>
-  </si>
-  <si>
-    <t>HE50 3</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/FF300393C_e5011223-6c02-4664-94da-5d2a6b0a2d8e.jpg?v=1760959543</t>
-  </si>
-  <si>
-    <t>FilterFinder FF300393C Compressed Air Filter | Replaces the Hi-Line HE50-3</t>
-  </si>
-  <si>
-    <t>he50-3-1</t>
-  </si>
-  <si>
-    <t>Style: Compressed Air Filter, Media: Polyester Needle Felt, Outer Diameter: 50.0 mm, Inner Diameter: 24.0 mm, Length: 73.5 mm, Seal Material: Nitrile, Temperature Range: +1 - +80°C, Media Type: Polyester Needle Felt, Flow Direction: IN-OUT, Seal: Nitrile</t>
-  </si>
-  <si>
-    <t>FF300393C</t>
-  </si>
-  <si>
-    <t>he25-4</t>
-  </si>
-  <si>
-    <t>HE25 4</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/products/FF300385C-R_02711a0d-7b66-4738-b25b-e0a2b3136243.webp?v=1673370144</t>
-  </si>
-  <si>
-    <t>FilterFinder FF300386C Compressed Air Filter | Replaces the Hi-Line HE25-4</t>
-  </si>
-  <si>
-    <t>he25-4-1</t>
-  </si>
-  <si>
-    <t>Style: Compressed Air Filter, Media: Polyester Needle Felt, Outer Diameter: 50.0 mm, Inner Diameter: 24.0 mm, Length: 50.0 mm, Seal Material: Nitrile, Temperature Range: +1 - +80°C, Media Type: Polyester Needle Felt, Flow Direction: IN-OUT, Seal: Nitrile</t>
-  </si>
-  <si>
-    <t>FF300386C</t>
-  </si>
-  <si>
-    <t>he25-3</t>
-  </si>
-  <si>
-    <t>HE25 3</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/products/FF300385C-R_15384020-b5c9-4190-ba11-8f8f8f1776e2.webp?v=1673370139</t>
-  </si>
-  <si>
-    <t>FilterFinder FF300385C Compressed Air Filter | Replaces the Hi-Line HE25-3</t>
-  </si>
-  <si>
-    <t>he25-3-1</t>
-  </si>
-  <si>
-    <t>FF300385C</t>
-  </si>
-  <si>
-    <t>Germany</t>
-  </si>
-  <si>
-    <t>Variant Metafield: custom.hs_code [single_line_text_field]</t>
-  </si>
-  <si>
-    <t>Variant Metafield: custom.country_of_origin [single_line_text_field]</t>
-  </si>
-  <si>
-    <t>Variant Metafield: custom.vendor [single_line_text_field]</t>
-  </si>
-  <si>
-    <t>hfl92001</t>
-  </si>
-  <si>
-    <t>HFL92001</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/p761490.700.700_76429a41-6dd3-4f01-a3be-47ef251b2e95.jpg?v=1762281289</t>
-  </si>
-  <si>
-    <t>Donaldson P761490 Hydraulic Filter, Cartridge | Replaces the Argo-Hytos HFL92001</t>
-  </si>
-  <si>
-    <t>hfl92001-1</t>
-  </si>
-  <si>
-    <t>8421.29.80.90</t>
-  </si>
-  <si>
-    <t>Italy</t>
-  </si>
-  <si>
-    <t>Genuine Donaldson P761490 Hydraulic Filter, Cartridge is designed to provide superior protection for your hydraulic system, effectively capturing contaminants to ensure clean fluid circulation. With high-quality filtration media, it extends equipment life, improves operational efficiency, and maintains fluid cleanliness even in the most demanding environments. Built for industrial, agricultural, and heavy-duty applications, this filter offers excellent dirt-holding capacity and flow efficiency. Its easy installation and maintenance help reduce downtime, making it a reliable choice for keeping hydraulic systems running smoothly.</t>
-  </si>
-  <si>
-    <t>Style: Special Filter, Media: Cellulose, Efficiency 1: 25µ @ β2, Outer Diameter: 109.0 mm, Inner Diameter: 19.0 mm, Length: 277.5 mm, Seal Material: Nitrile, Temperature Range: -30 - +100°C, Efficiency 1 The efficiency of the element is shown using the Micron (µ) and Beta (β) ratings. The micron rating indicates the size of the particle being filtered and the beta rating the efficiency , calculated as 1/β. E.g. a rating of β200 will be 99.5% efficient whereas β1000 would be 99.9%.: 25µ @ β2, Media Type: Cellulose, Flow Direction: OUT-IN, Seal: Nitrile</t>
-  </si>
-  <si>
-    <t>P761490</t>
-  </si>
-  <si>
-    <t>0.5 kg</t>
-  </si>
-  <si>
-    <t>0.0058 m³</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/md-a0c9e004-1459-42ad-a8c2-320cdf9cded1_a5132323-2482-4394-8cd6-541d30a3af8f.jpg?v=1762281289</t>
-  </si>
-  <si>
-    <t>HiFi Filter SH 52102 Special Filter | Replaces the Argo-Hytos HFL92001</t>
-  </si>
-  <si>
-    <t>hfl92001-2</t>
-  </si>
-  <si>
-    <t>8421.99.90</t>
-  </si>
-  <si>
-    <t>France</t>
-  </si>
-  <si>
-    <t>Genuine HiFi Filter SH 52102 Hydraulic Filter. Engineered to protect and optimize the performance of hydraulic systems, this filter delivers exceptional contamination control. Premium filter media captures fine particles and debris that could compromise system integrity, helping to extend the lifespan of critical hydraulic components. By maintaining fluid cleanliness, it reduces wear and tear while supporting consistent pressure levels throughout the system. Perfect for a wide range of hydraulic applications—from industrial machinery to heavy-duty equipment—this filter provides reliable performance even under high-pressure conditions. Its robust construction ensures long-lasting durability, helping to minimize downtime and maintenance costs while maximizing operational efficiency.</t>
-  </si>
-  <si>
-    <t>Style: HYDRAULIC FILTER, Dimension 1 (D1): 109.0 mm, Dimension 2 (D2): 99.5 mm, Dimension 3 (D3): 19.0 mm, Height 1 (H1): 276.0 mm, Height 2 (H2): 255.0 mm, Height 3 (H3): 231.0 mm, Efficiency 1 The efficiency of the element is shown using the Micron (µ) and Beta (β) ratings. The micron rating indicates the size of the particle being filtered and the beta rating the efficiency , calculated as 1/β. E.g. a rating of β200 will be 99.5% efficient whereas β1000 would be 99.9%.: 25µ @ β2, Outer Diameter: 109.0 mm, Inner Diameter: 19.0 mm, Length: 277.5 mm, Media Type: Cellulose, Flow Direction: OUT-IN, Seal: Nitrile, Temperature Range: -30 - +100°C</t>
-  </si>
-  <si>
-    <t>SH 52102</t>
-  </si>
-  <si>
-    <t>0.62 kg</t>
-  </si>
-  <si>
-    <t>0.0045 m³</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/placeholder_05c9f458-190b-4228-8de0-e336cc07ce35.png?v=1762281289</t>
-  </si>
-  <si>
-    <t>Filtrec WP459 Special Filter | Replaces the Argo-Hytos HFL92001</t>
-  </si>
-  <si>
-    <t>hfl92001-3</t>
-  </si>
-  <si>
-    <t>Genuine Filtrec WP459. This Filtrec element is designed to meet or exceed the quality and performance of brand OEM’s ensuring superior filtration performance and long-lasting durability. Engineered with their high performance media and a durable design, the WP459 provides reliable and consistent performance over its lifespan, even in harsh operating environments. When you order from FilterFinder, you can trust that you are getting a reliable and high-quality replacement filter that will keep your system running smoothly.</t>
-  </si>
-  <si>
-    <t>WP459</t>
-  </si>
-  <si>
-    <t>0.61 kg</t>
-  </si>
-  <si>
-    <t>0.0033 m³</t>
-  </si>
-  <si>
-    <t>as025-01</t>
-  </si>
-  <si>
-    <t>AS025 01</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/md-ead133b0-35b1-4d4e-99bd-0ca39f12dc1e_42cf2fc6-8749-49b5-8e24-0f9e38f315d7.jpg?v=1762275856</t>
-  </si>
-  <si>
-    <t>HiFi Filter SH 77007 Suction Strainer | Replaces the Argo-Hytos AS025-01</t>
-  </si>
-  <si>
-    <t>as025-01-2</t>
-  </si>
-  <si>
-    <t>Genuine HiFi Filter SH 77007 Hydraulic Filter. Engineered to protect and optimize the performance of hydraulic systems, this filter delivers exceptional contamination control. Premium filter media captures fine particles and debris that could compromise system integrity, helping to extend the lifespan of critical hydraulic components. By maintaining fluid cleanliness, it reduces wear and tear while supporting consistent pressure levels throughout the system. Perfect for a wide range of hydraulic applications—from industrial machinery to heavy-duty equipment—this filter provides reliable performance even under high-pressure conditions. Its robust construction ensures long-lasting durability, helping to minimize downtime and maintenance costs while maximizing operational efficiency.</t>
-  </si>
-  <si>
-    <t>Style: HYDRAULIC FILTER, Dimension 1 (D1): 63.0 mm, Dimension 2 (D2): 36.0 mm, Thread 1 (D7): 3/4"-BSP, Height 1 (H1): 109.0 mm, Height 2 (H2): 101.0 mm, Efficiency 1 The efficiency of the element is shown using the Micron (µ) and Beta (β) ratings. The micron rating indicates the size of the particle being filtered and the beta rating the efficiency , calculated as 1/β. E.g. a rating of β200 will be 99.5% efficient whereas β1000 would be 99.9%.: 125µ, Outer Diameter: 64.0 mm, Length: 109.0 mm, Media Type: Wire Mesh, Flow Direction: OUT-IN, Thread: 3/4" BSP, Collapse Pressure: 1 BAR, Temperature Range: -30 - +100°C</t>
-  </si>
-  <si>
-    <t>SH 77007</t>
-  </si>
-  <si>
-    <t>0.16 kg</t>
-  </si>
-  <si>
-    <t>0.0009 m³</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/Argo-Hytos_Placeholder_2c74e0fd-88a7-45d4-81a6-9fd71db5072e.jpg?v=1762275856</t>
-  </si>
-  <si>
-    <t>Argo Hytos AS02501 Suction Strainer</t>
-  </si>
-  <si>
-    <t>as025-01-3</t>
-  </si>
-  <si>
-    <t>Original Argo-Hytos AS02501 filter. Benefits - Reliable oil cleanliness and permanent protection of sensitive components over the entire operating life. - Good cold start performance, i.e. closed bypass valve even at low temperatures. Lower energy consumption results in lower operating costs and conserves resources. - Longer maintenance intervals and thus improved productivity and economic efficiency. - Excellent differential pressure stability, ensuring filtration stability by avoiding damage to the filter bellows. - High flow fatigue strength which guarantee of oil cleanliness even with strongly alternating flow loads.</t>
-  </si>
-  <si>
-    <t>Style: Suction Strainer, Media: Wire Mesh, Efficiency 1: 125µ, Outer Diameter: 64.0 mm, Length: 109.0 mm, Thread: 3/4" BSP, Δ Collapse Pressure: 1 bar, Temperature Range: -30 - +100°C, Efficiency 1 The efficiency of the element is shown using the Micron (µ) and Beta (β) ratings. The micron rating indicates the size of the particle being filtered and the beta rating the efficiency , calculated as 1/β. E.g. a rating of β200 will be 99.5% efficient whereas β1000 would be 99.9%.: 125µ, Media Type: Wire Mesh, Flow Direction: OUT-IN, Collapse Pressure: 1 BAR</t>
-  </si>
-  <si>
-    <t>AS02501</t>
-  </si>
-  <si>
-    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/0025_s_125_w_n165585_i2372437_54eabc50-8f5a-4f88-a2c5-0767c9f6390e.jpg?v=1762275856</t>
-  </si>
-  <si>
-    <t>Hydac 0025 S 125 W Suction Strainer | Replaces the Argo-Hytos AS025-01</t>
-  </si>
-  <si>
-    <t>as025-01-4</t>
-  </si>
-  <si>
-    <t>Genuine Hydac 0025 S 125 W Suction Strainer. Built to HYDAC’s OEM specifications and quality standards, this genuine part offers reliable performance, long service life and a precise fit. It’s suitable for a wide range of hydraulic and process applications, helping protect equipment, reduce downtime and maintain system cleanliness. For best results, match the part code to your equipment manual and verify key dimensions and ratings (size, connection, filtration grade/flow) before installation.</t>
-  </si>
-  <si>
-    <t>0025 S 125 W</t>
-  </si>
-  <si>
     <t>test</t>
   </si>
   <si>
-    <t>Compressed Air Filters, test</t>
-  </si>
-  <si>
-    <t>test, ff1225</t>
-  </si>
-  <si>
-    <t>Argo Hytos, ff1225, test</t>
-  </si>
-  <si>
-    <t>Argo Hytos, test</t>
+    <t>270l110a</t>
+  </si>
+  <si>
+    <t>270L110A</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/md-ecbdeaf4-3809-4bd7-9655-84f4e8f1ee1c_11ab6aeb-ef0f-48b7-aded-283abe63b831.jpg?v=1764690896</t>
+  </si>
+  <si>
+    <t>HiFi Filter SH 56261 Pressure Filter | Replaces the Fairey Arlon 270L110A</t>
+  </si>
+  <si>
+    <t>270l110a-1</t>
+  </si>
+  <si>
+    <t>Genuine HiFi Filter SH 56261 Hydraulic Filter. Engineered to protect and optimize the performance of hydraulic systems, this filter delivers exceptional contamination control. Premium filter media captures fine particles and debris that could compromise system integrity, helping to extend the lifespan of critical hydraulic components. By maintaining fluid cleanliness, it reduces wear and tear while supporting consistent pressure levels throughout the system. Perfect for a wide range of hydraulic applications—from industrial machinery to heavy-duty equipment—this filter provides reliable performance even under high-pressure conditions. Its robust construction ensures long-lasting durability, helping to minimize downtime and maintenance costs while maximizing operational efficiency.</t>
+  </si>
+  <si>
+    <t>Style: HYDRAULIC FILTER, Dimension 1 (D1): 73.0 mm, Dimension 2 (D2): 32.0 mm, Dimension 3 (D3): 31.0 mm, Height 1 (H1): 102.0 mm, Height 2 (H2): 98.0 mm, Height 3 (H3): 95.0 mm, Efficiency 1 The efficiency of the element is shown using the Micron (µ) and Beta (β) ratings. The micron rating indicates the size of the particle being filtered and the beta rating the efficiency , calculated as 1/β. E.g. a rating of β200 will be 99.5% efficient whereas β1000 would be 99.9%.: 20µ @ β200, Efficiency 2: 22µ @ β1000, Outer Diameter: 73.6 mm, Inner Diameter: 32.0 mm, Length: 99.0 mm, Media Type: Glass Fiber, Flow Direction: OUT-IN, Collapse Pressure: 25 BAR, Seal: Nitrile, Temperature Range: -30 - +100°C</t>
+  </si>
+  <si>
+    <t>SH 56261</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/products/FF203284B_76c4ed4f-cced-4090-87b0-f05d7dabf858.jpg?v=1764690896</t>
+  </si>
+  <si>
+    <t>MicroFit® UltraGen III MFHLP31079 Pressure Filter | Replaces the Fairey Arlon 270L110A</t>
+  </si>
+  <si>
+    <t>270l110a-2</t>
+  </si>
+  <si>
+    <t>The MICROFIT® UltraGen III MFHLP31079 is the MICROFIT® approved replacement to the Fairey Arlon 270L110A. Engineered and manufactured in Great Britain the MFHLP31079 is designed to meet or exceed the quality and performance of OEM quality standards, ensuring superior filtration performance and the longest possible filter life. Building on over 50 years of filtration expertise, the UltraGen III series is the third generation of MICROFIT® filter media, delivering exceptional efficiency and reliability. FilterFinder is an approved distributor of MICROFIT® filters. With expert product knowledge, dedicated support, and a large stock availability, FilterFinder ensures you receive the parts you need when you need them, every time.</t>
+  </si>
+  <si>
+    <t>Style: Pressure Filter, Media: Glass Fiber, Efficiency 1: 20µ @ β200, Efficiency 2: 22µ @ β1000, Outer Diameter: 73.6 mm, Inner Diameter: 32.0 mm, Length: 99.0 mm, Δ Collapse Pressure: 25 bar, Seal Material: Nitrile, Temperature Range: -30 - +100°C, Efficiency 1 The efficiency of the element is shown using the Micron (µ) and Beta (β) ratings. The micron rating indicates the size of the particle being filtered and the beta rating the efficiency , calculated as 1/β. E.g. a rating of β200 will be 99.5% efficient whereas β1000 would be 99.9%.: 20µ @ β200, Media Type: Glass Fiber, Flow Direction: OUT-IN, Collapse Pressure: 25 BAR, Seal: Nitrile</t>
+  </si>
+  <si>
+    <t>MFHLP31079</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/p173030.700.700_935956e8-1782-47e3-9fc7-d04a35431fce.jpg?v=1764690896</t>
+  </si>
+  <si>
+    <t>Donaldson P173030 Hydraulic Filter, Cartridge | Replaces the Fairey Arlon 270L110A</t>
+  </si>
+  <si>
+    <t>270l110a-3</t>
+  </si>
+  <si>
+    <t>Genuine Donaldson P173030 Hydraulic Filter, Cartridge is designed to provide superior protection for your hydraulic system, effectively capturing contaminants to ensure clean fluid circulation. With high-quality filtration media, it extends equipment life, improves operational efficiency, and maintains fluid cleanliness even in the most demanding environments. Built for industrial, agricultural, and heavy-duty applications, this filter offers excellent dirt-holding capacity and flow efficiency. Its easy installation and maintenance help reduce downtime, making it a reliable choice for keeping hydraulic systems running smoothly.</t>
+  </si>
+  <si>
+    <t>P173030</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/D910_77ad6b58-6985-4483-9566-668ebf6e00be.jpg?v=1764690896</t>
+  </si>
+  <si>
+    <t>Filtrec D920G25A Pressure Filter | Replaces the Fairey Arlon 270L110A</t>
+  </si>
+  <si>
+    <t>270l110a-4</t>
+  </si>
+  <si>
+    <t>Genuine Filtrec D920G25A. This Filtrec element is designed to meet or exceed the quality and performance of brand OEM’s ensuring superior filtration performance and long-lasting durability. Engineered with their high performance media and a durable design, the D920G25A provides reliable and consistent performance over its lifespan, even in harsh operating environments. When you order from FilterFinder, you can trust that you are getting a reliable and high-quality replacement filter that will keep your system running smoothly.</t>
+  </si>
+  <si>
+    <t>D920G25A</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/HF30714_b98529f8-c59f-4616-af96-93c7444caa8b.jpg?v=1764690896</t>
+  </si>
+  <si>
+    <t>Fleetguard HF30714 Hydraulic Filters | Replaces the Fairey Arlon 270L110A</t>
+  </si>
+  <si>
+    <t>270l110a-5</t>
+  </si>
+  <si>
+    <t>Fleetguard® HF30714 hydraulic cartridge filter with synthetic media is designed to help keep your precision hydraulic systems running as intended, providing a solution for various applications.  This filter meets or exceeds the equipment OEM quality and performance and is the first aftermarket replacement available on the market today, bringing your operation top-quality performance and an overall unbeatable total cost of ownership.</t>
+  </si>
+  <si>
+    <t>HF30714</t>
+  </si>
+  <si>
+    <t>270l201a</t>
+  </si>
+  <si>
+    <t>270L201A</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/FF203286B_0e7cd06a-33d3-4249-b2af-cef48cbe7cea.jpg?v=1764692272</t>
+  </si>
+  <si>
+    <t>MicroFit® UltraGen III MFHLP31235 Pressure Filter | Replaces the Fairey Arlon 270L201A</t>
+  </si>
+  <si>
+    <t>270l201a-1</t>
+  </si>
+  <si>
+    <t>The MICROFIT® UltraGen III MFHLP31235 is the MICROFIT® approved replacement to the Fairey Arlon 270L201A. Engineered and manufactured in Great Britain the MFHLP31235 is designed to meet or exceed the quality and performance of OEM quality standards, ensuring superior filtration performance and the longest possible filter life. Building on over 50 years of filtration expertise, the UltraGen III series is the third generation of MICROFIT® filter media, delivering exceptional efficiency and reliability. FilterFinder is an approved distributor of MICROFIT® filters. With expert product knowledge, dedicated support, and a large stock availability, FilterFinder ensures you receive the parts you need when you need them, every time.</t>
+  </si>
+  <si>
+    <t>Style: Pressure Filter, Media: Glass Fiber, Efficiency 1: 5µ @ β200, Efficiency 2: 7µ @ β1000, Outer Diameter: 73.6 mm, Inner Diameter: 32.0 mm, Length: 232.0 mm, Δ Collapse Pressure: 25 bar, Seal Material: Nitrile, Temperature Range: -30 - +100°C, Efficiency 1 The efficiency of the element is shown using the Micron (µ) and Beta (β) ratings. The micron rating indicates the size of the particle being filtered and the beta rating the efficiency , calculated as 1/β. E.g. a rating of β200 will be 99.5% efficient whereas β1000 would be 99.9%.: 5µ @ β200, Media Type: Glass Fiber, Flow Direction: OUT-IN, Collapse Pressure: 25 BAR, Seal: Nitrile</t>
+  </si>
+  <si>
+    <t>MFHLP31235</t>
+  </si>
+  <si>
+    <t>1.23 kg</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/D921_d07b3597-3693-4e5e-acaa-2608aada60f0.jpg?v=1764692272</t>
+  </si>
+  <si>
+    <t>Filtrec D921G06A Pressure Filter | Replaces the Fairey Arlon 270L201A</t>
+  </si>
+  <si>
+    <t>270l201a-2</t>
+  </si>
+  <si>
+    <t>Genuine Filtrec D921G06A. This Filtrec element is designed to meet or exceed the quality and performance of brand OEM’s ensuring superior filtration performance and long-lasting durability. Engineered with their high performance media and a durable design, the D921G06A provides reliable and consistent performance over its lifespan, even in harsh operating environments. When you order from FilterFinder, you can trust that you are getting a reliable and high-quality replacement filter that will keep your system running smoothly.</t>
+  </si>
+  <si>
+    <t>D921G06A</t>
+  </si>
+  <si>
+    <t>0.57 kg</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/p173032.700.700_babc10cc-0aff-415b-80ba-2b3ee74c6b87.jpg?v=1764692272</t>
+  </si>
+  <si>
+    <t>Donaldson P173032 Hydraulic Filter, Cartridge | Replaces the Fairey Arlon 270L201A</t>
+  </si>
+  <si>
+    <t>270l201a-3</t>
+  </si>
+  <si>
+    <t>Genuine Donaldson P173032 Hydraulic Filter, Cartridge is designed to provide superior protection for your hydraulic system, effectively capturing contaminants to ensure clean fluid circulation. With high-quality filtration media, it extends equipment life, improves operational efficiency, and maintains fluid cleanliness even in the most demanding environments. Built for industrial, agricultural, and heavy-duty applications, this filter offers excellent dirt-holding capacity and flow efficiency. Its easy installation and maintenance help reduce downtime, making it a reliable choice for keeping hydraulic systems running smoothly.</t>
+  </si>
+  <si>
+    <t>P173032</t>
+  </si>
+  <si>
+    <t>https://cdn.shopify.com/s/files/1/0592/2648/8986/files/md-0eacc112-2fbd-4242-8e20-41a570f7116a_caefb2a6-2dcb-493a-a313-4063f8b6810b.jpg?v=1764692272</t>
+  </si>
+  <si>
+    <t>HiFi Filter SH 53012 Pressure Filter | Replaces the Fairey Arlon 270L201A</t>
+  </si>
+  <si>
+    <t>270l201a-4</t>
+  </si>
+  <si>
+    <t>Genuine HiFi Filter SH 53012 Hydraulic Filter. Engineered to protect and optimize the performance of hydraulic systems, this filter delivers exceptional contamination control. Premium filter media captures fine particles and debris that could compromise system integrity, helping to extend the lifespan of critical hydraulic components. By maintaining fluid cleanliness, it reduces wear and tear while supporting consistent pressure levels throughout the system. Perfect for a wide range of hydraulic applications—from industrial machinery to heavy-duty equipment—this filter provides reliable performance even under high-pressure conditions. Its robust construction ensures long-lasting durability, helping to minimize downtime and maintenance costs while maximizing operational efficiency.</t>
+  </si>
+  <si>
+    <t>SH 53012</t>
+  </si>
+  <si>
+    <t>Test, ff1225</t>
   </si>
 </sst>
 </file>
@@ -827,8 +863,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BF12"/>
+  <dimension ref="A1:BF13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="24" max="24" width="9.08984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -982,10 +1021,10 @@
         <v>49</v>
       </c>
       <c r="AY1" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="AZ1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="BA1" t="s">
         <v>50</v>
@@ -1003,7 +1042,7 @@
         <v>54</v>
       </c>
       <c r="BF1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:58" x14ac:dyDescent="0.35">
@@ -1017,7 +1056,7 @@
         <v>57</v>
       </c>
       <c r="G2" t="s">
-        <v>151</v>
+        <v>104</v>
       </c>
       <c r="H2" t="s">
         <v>56</v>
@@ -1059,7 +1098,7 @@
         <v>61</v>
       </c>
       <c r="AM2">
-        <v>11800</v>
+        <v>7100</v>
       </c>
       <c r="AR2" t="s">
         <v>65</v>
@@ -1076,25 +1115,40 @@
       <c r="AV2" t="s">
         <v>68</v>
       </c>
+      <c r="AY2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>71</v>
+      </c>
       <c r="BB2" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="BC2" t="s">
-        <v>70</v>
+        <v>57</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>72</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
         <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="G3" t="s">
-        <v>152</v>
+        <v>104</v>
       </c>
       <c r="H3" t="s">
         <v>56</v>
@@ -1109,7 +1163,7 @@
         <v>60</v>
       </c>
       <c r="T3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="U3" t="s">
         <v>56</v>
@@ -1124,19 +1178,19 @@
         <v>62</v>
       </c>
       <c r="AA3" t="s">
+        <v>75</v>
+      </c>
+      <c r="AG3">
+        <v>2</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>76</v>
+      </c>
+      <c r="AJ3" t="s">
         <v>74</v>
       </c>
-      <c r="AG3">
-        <v>1</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>75</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>73</v>
-      </c>
       <c r="AM3">
-        <v>11800</v>
+        <v>8400</v>
       </c>
       <c r="AR3" t="s">
         <v>65</v>
@@ -1153,25 +1207,37 @@
       <c r="AV3" t="s">
         <v>68</v>
       </c>
+      <c r="AY3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>78</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>79</v>
+      </c>
       <c r="BB3" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="BC3" t="s">
-        <v>76</v>
+        <v>80</v>
+      </c>
+      <c r="BD3" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>105</v>
       </c>
       <c r="B4" t="s">
         <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="G4" t="s">
-        <v>152</v>
+        <v>112</v>
       </c>
       <c r="H4" t="s">
         <v>56</v>
@@ -1186,7 +1252,7 @@
         <v>60</v>
       </c>
       <c r="T4" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="U4" t="s">
         <v>56</v>
@@ -1201,19 +1267,19 @@
         <v>62</v>
       </c>
       <c r="AA4" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="AG4">
         <v>1</v>
       </c>
       <c r="AH4" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="AJ4" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="AM4">
-        <v>7200</v>
+        <v>11800</v>
       </c>
       <c r="AR4" t="s">
         <v>65</v>
@@ -1231,24 +1297,24 @@
         <v>68</v>
       </c>
       <c r="BB4" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="BC4" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
         <v>56</v>
       </c>
       <c r="C5" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="G5" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
       <c r="H5" t="s">
         <v>56</v>
@@ -1263,7 +1329,7 @@
         <v>60</v>
       </c>
       <c r="T5" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="U5" t="s">
         <v>56</v>
@@ -1278,19 +1344,19 @@
         <v>62</v>
       </c>
       <c r="AA5" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
       <c r="AG5">
         <v>1</v>
       </c>
       <c r="AH5" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
       <c r="AJ5" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="AM5">
-        <v>5400</v>
+        <v>3100</v>
       </c>
       <c r="AR5" t="s">
         <v>65</v>
@@ -1307,25 +1373,40 @@
       <c r="AV5" t="s">
         <v>68</v>
       </c>
+      <c r="AY5" t="s">
+        <v>69</v>
+      </c>
+      <c r="AZ5" t="s">
+        <v>70</v>
+      </c>
+      <c r="BA5" t="s">
+        <v>118</v>
+      </c>
       <c r="BB5" t="s">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="BC5" t="s">
+        <v>120</v>
+      </c>
+      <c r="BD5" t="s">
         <v>90</v>
+      </c>
+      <c r="BE5" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
         <v>56</v>
       </c>
       <c r="C6" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="G6" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="H6" t="s">
         <v>56</v>
@@ -1340,7 +1421,7 @@
         <v>60</v>
       </c>
       <c r="T6" t="s">
-        <v>93</v>
+        <v>121</v>
       </c>
       <c r="U6" t="s">
         <v>56</v>
@@ -1355,19 +1436,19 @@
         <v>62</v>
       </c>
       <c r="AA6" t="s">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AG6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH6" t="s">
-        <v>95</v>
+        <v>123</v>
       </c>
       <c r="AJ6" t="s">
-        <v>93</v>
+        <v>121</v>
       </c>
       <c r="AM6">
-        <v>5400</v>
+        <v>3800</v>
       </c>
       <c r="AR6" t="s">
         <v>65</v>
@@ -1384,25 +1465,40 @@
       <c r="AV6" t="s">
         <v>68</v>
       </c>
+      <c r="AY6" t="s">
+        <v>69</v>
+      </c>
+      <c r="AZ6" t="s">
+        <v>101</v>
+      </c>
+      <c r="BA6" t="s">
+        <v>124</v>
+      </c>
       <c r="BB6" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
       <c r="BC6" t="s">
+        <v>126</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>93</v>
+      </c>
+      <c r="BE6" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
         <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="G7" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="H7" t="s">
         <v>56</v>
@@ -1417,7 +1513,7 @@
         <v>60</v>
       </c>
       <c r="T7" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="U7" t="s">
         <v>56</v>
@@ -1432,19 +1528,19 @@
         <v>62</v>
       </c>
       <c r="AA7" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="AG7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH7" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="AJ7" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="AM7">
-        <v>6000</v>
+        <v>4100</v>
       </c>
       <c r="AR7" t="s">
         <v>65</v>
@@ -1462,39 +1558,39 @@
         <v>68</v>
       </c>
       <c r="AY7" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="AZ7" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="BA7" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="BB7" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="BC7" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="BD7" t="s">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="BE7" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B8" t="s">
         <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="G8" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="H8" t="s">
         <v>56</v>
@@ -1509,7 +1605,7 @@
         <v>60</v>
       </c>
       <c r="T8" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="U8" t="s">
         <v>56</v>
@@ -1524,19 +1620,19 @@
         <v>62</v>
       </c>
       <c r="AA8" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="AG8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AH8" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="AJ8" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="AM8">
-        <v>5400</v>
+        <v>4100</v>
       </c>
       <c r="AR8" t="s">
         <v>65</v>
@@ -1554,39 +1650,39 @@
         <v>68</v>
       </c>
       <c r="AY8" t="s">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="AZ8" t="s">
-        <v>117</v>
+        <v>84</v>
       </c>
       <c r="BA8" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="BB8" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="BC8" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="BD8" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="BE8" t="s">
-        <v>122</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B9" t="s">
         <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="G9" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="H9" t="s">
         <v>56</v>
@@ -1601,7 +1697,7 @@
         <v>60</v>
       </c>
       <c r="T9" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="U9" t="s">
         <v>56</v>
@@ -1616,19 +1712,19 @@
         <v>62</v>
       </c>
       <c r="AA9" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="AG9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AH9" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="AJ9" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="AM9">
-        <v>0</v>
+        <v>4700</v>
       </c>
       <c r="AR9" t="s">
         <v>65</v>
@@ -1646,39 +1742,39 @@
         <v>68</v>
       </c>
       <c r="AY9" t="s">
-        <v>116</v>
+        <v>83</v>
       </c>
       <c r="AZ9" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="BA9" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="BB9" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="BC9" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="BD9" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="BE9" t="s">
-        <v>129</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="B10" t="s">
         <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="G10" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="H10" t="s">
         <v>56</v>
@@ -1693,7 +1789,7 @@
         <v>60</v>
       </c>
       <c r="T10" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="U10" t="s">
         <v>56</v>
@@ -1708,19 +1804,19 @@
         <v>62</v>
       </c>
       <c r="AA10" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="AG10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH10" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="AJ10" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="AM10">
-        <v>2500</v>
+        <v>7000</v>
       </c>
       <c r="AR10" t="s">
         <v>65</v>
@@ -1738,39 +1834,39 @@
         <v>68</v>
       </c>
       <c r="AY10" t="s">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="AZ10" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="BA10" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="BB10" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="BC10" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="BD10" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="BE10" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="B11" t="s">
         <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="G11" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="H11" t="s">
         <v>56</v>
@@ -1785,7 +1881,7 @@
         <v>60</v>
       </c>
       <c r="T11" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="U11" t="s">
         <v>56</v>
@@ -1800,19 +1896,19 @@
         <v>62</v>
       </c>
       <c r="AA11" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="AG11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH11" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="AJ11" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="AM11">
-        <v>3600</v>
+        <v>7700</v>
       </c>
       <c r="AR11" t="s">
         <v>65</v>
@@ -1830,33 +1926,39 @@
         <v>68</v>
       </c>
       <c r="AY11" t="s">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="AZ11" t="s">
+        <v>84</v>
+      </c>
+      <c r="BA11" t="s">
+        <v>154</v>
+      </c>
+      <c r="BB11" t="s">
+        <v>148</v>
+      </c>
+      <c r="BC11" t="s">
+        <v>155</v>
+      </c>
+      <c r="BD11" t="s">
+        <v>156</v>
+      </c>
+      <c r="BE11" t="s">
         <v>97</v>
-      </c>
-      <c r="BA11" t="s">
-        <v>143</v>
-      </c>
-      <c r="BB11" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC11" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="B12" t="s">
         <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="G12" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="H12" t="s">
         <v>56</v>
@@ -1871,7 +1973,7 @@
         <v>60</v>
       </c>
       <c r="T12" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="U12" t="s">
         <v>56</v>
@@ -1886,19 +1988,19 @@
         <v>62</v>
       </c>
       <c r="AA12" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="AG12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AH12" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="AJ12" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="AM12">
-        <v>4600</v>
+        <v>8600</v>
       </c>
       <c r="AR12" t="s">
         <v>65</v>
@@ -1916,19 +2018,117 @@
         <v>68</v>
       </c>
       <c r="AY12" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="AZ12" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="BA12" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="BB12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="BC12" t="s">
-        <v>150</v>
+        <v>161</v>
+      </c>
+      <c r="BD12" t="s">
+        <v>94</v>
+      </c>
+      <c r="BE12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:58" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>142</v>
+      </c>
+      <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
+        <v>143</v>
+      </c>
+      <c r="G13" t="s">
+        <v>167</v>
+      </c>
+      <c r="H13" t="s">
+        <v>56</v>
+      </c>
+      <c r="I13" t="s">
+        <v>58</v>
+      </c>
+      <c r="J13" t="s">
+        <v>59</v>
+      </c>
+      <c r="L13" t="s">
+        <v>60</v>
+      </c>
+      <c r="T13" t="s">
+        <v>162</v>
+      </c>
+      <c r="U13" t="s">
+        <v>56</v>
+      </c>
+      <c r="V13">
+        <v>1</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG13">
+        <v>4</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>164</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>162</v>
+      </c>
+      <c r="AM13">
+        <v>10500</v>
+      </c>
+      <c r="AR13" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS13" t="s">
+        <v>66</v>
+      </c>
+      <c r="AT13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AU13" t="s">
+        <v>59</v>
+      </c>
+      <c r="AV13" t="s">
+        <v>68</v>
+      </c>
+      <c r="AY13" t="s">
+        <v>69</v>
+      </c>
+      <c r="AZ13" t="s">
+        <v>70</v>
+      </c>
+      <c r="BA13" t="s">
+        <v>165</v>
+      </c>
+      <c r="BB13" t="s">
+        <v>148</v>
+      </c>
+      <c r="BC13" t="s">
+        <v>166</v>
+      </c>
+      <c r="BD13" t="s">
+        <v>92</v>
+      </c>
+      <c r="BE13" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>